<commit_message>
fix(anotacion): corrige el ejemplo del esquema y lo alinea con la leyenda
El ejemplo de fila completa usaba "Gobierno nacional" como actor_objetivo,
valor que no existe en la lista cerrada de 9 opciones; queda en
"Gobierno / Ejecutivo".

La misma oracion de ejemplo estaba anotada distinto en los dos documentos
que ve el anotador: la leyenda del corpus marcaba palabra_subjetiva en TRUE
con span "impuso" y esquemas_anotacion en FALSE. Se adopta la version de la
leyenda, que es la correcta por definicion de la categoria, y la Tabla 2
pasa a mostrar los 3 hallazgos de la oracion en vez de 2.
</commit_message>
<xml_diff>
--- a/data/corpus/esquemas_anotacion.xlsx
+++ b/data/corpus/esquemas_anotacion.xlsx
@@ -1037,7 +1037,7 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE / span: "impuso"</t>
         </is>
       </c>
     </row>
@@ -1603,39 +1603,39 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
+          <t>TRUE ("impuso")</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>TRUE ("polémica")</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>TRUE ("polémica")</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>TRUE ("sabiendo que afectaría directamente a la clase media")</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>TRUE ("sabiendo que afectaría directamente a la clase media")</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="N34" s="2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
           <t>perjudica</t>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>Gobierno nacional</t>
+          <t>Gobierno / Ejecutivo</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
@@ -1747,7 +1747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="7" min="1" max="1"/>
@@ -2148,6 +2148,48 @@
         </is>
       </c>
       <c r="I20" s="15" t="n"/>
+    </row>
+    <row r="21" ht="118.5" customHeight="1" s="7">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>ART_0231</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>ART_0231_S07</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>El Gobierno impuso la polémica reforma tributaria pese a las advertencias de los gremios, sabiendo que afectaría directamente a la clase media.</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>impuso</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>lexico</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>perjudica</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Gobierno / Ejecutivo</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>